<commit_message>
blue icon file 2
</commit_message>
<xml_diff>
--- a/docs/tasks-lambda.xlsx
+++ b/docs/tasks-lambda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\einav\clone_here\Lambda\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C4B9EB-AC2B-4BDD-8F1E-BB7F7C92A1BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5537CD4A-429E-4F5E-963A-0703E6871F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{64494733-B6F9-48B6-9193-F7C7FF2B1841}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>הוספה של אופציה להוסיף שאלות כלליות (לאו דווקא ממבחן) - רבות ברירה, שאלות פתוחות</t>
   </si>
@@ -183,6 +183,27 @@
   </si>
   <si>
     <t>בשאלות שהן flash cards לא צריך שיהיה community solutions</t>
+  </si>
+  <si>
+    <t>generate questions</t>
+  </si>
+  <si>
+    <t>אני רוצה שיהיה משתמש admin שאוסיף ישירות בsupabase שיכול לערוך את כל התוכן באתר</t>
+  </si>
+  <si>
+    <t>אופציה להעלות תמונות בכרטיסי תוכן - צריך להיות הכי יעיל שאפשר ולכווץ את התמונות כמה שיותר. תן לי תוכנית קודם. שימוש בsupabase storage.</t>
+  </si>
+  <si>
+    <t>שדרך המשתמש Admin יהיה אפשר לשלוח הודעות למשתמשי האתר שיקפצו להם בלוח הודעות</t>
+  </si>
+  <si>
+    <t>תגובות בעמוד של הגרסה של הקורס</t>
+  </si>
+  <si>
+    <t>דירוג גרסה</t>
+  </si>
+  <si>
+    <t>שכפתור דיווח על טעות ישלח מייל לא רק לכותב הגרסה אלא גם אליי</t>
   </si>
 </sst>
 </file>
@@ -589,7 +610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ABCB3E3-AEE1-47E5-A283-0150B72CF279}">
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.45">
@@ -958,7 +979,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A44" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B44" t="s">
         <v>48</v>
@@ -968,20 +989,56 @@
       <c r="A45" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="B45" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A46" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="B46" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A47" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="B47" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A48" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="B48" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A49" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B49" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A50" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B50" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A51" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B51" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fork, community solutions, ,mail
</commit_message>
<xml_diff>
--- a/docs/tasks-lambda.xlsx
+++ b/docs/tasks-lambda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\einav\clone_here\Lambda\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6A5EE5-A49B-4CDA-A8A8-F0DFA2C66947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F995A4-B7D5-4E47-9AD1-B0F80BD06053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{64494733-B6F9-48B6-9193-F7C7FF2B1841}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>הוספה של אופציה להוסיף שאלות כלליות (לאו דווקא ממבחן) - רבות ברירה, שאלות פתוחות</t>
   </si>
@@ -210,6 +210,9 @@
   </si>
   <si>
     <t>בcontributions בפרופיל שיהיה קישור לcontribution. כרגע יש לגרסאות אבל לא לפתרונות</t>
+  </si>
+  <si>
+    <t>שיהיה אפשר לראות את הcommunity solutions רק כשעוברים לtab של הפתרון</t>
   </si>
 </sst>
 </file>
@@ -1017,7 +1020,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A48" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B48" t="s">
         <v>52</v>
@@ -1041,7 +1044,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A51" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B51" t="s">
         <v>55</v>
@@ -1049,7 +1052,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A52" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B52" t="s">
         <v>56</v>
@@ -1057,7 +1060,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A53" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B53" t="s">
         <v>57</v>
@@ -1065,7 +1068,10 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A54" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B54" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
fix: export practice service interfaces for TS build
</commit_message>
<xml_diff>
--- a/docs/tasks-lambda.xlsx
+++ b/docs/tasks-lambda.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\einav\clone_here\Lambda\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359C5C6F-1A66-4EB0-B64C-1A347D277837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44801C37-259E-4513-8374-D964EEA96DB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{64494733-B6F9-48B6-9193-F7C7FF2B1841}"/>
+    <workbookView xWindow="3247" yWindow="2138" windowWidth="16200" windowHeight="9307" xr2:uid="{64494733-B6F9-48B6-9193-F7C7FF2B1841}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A92" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B92" t="s">
         <v>96</v>

</xml_diff>

<commit_message>
leadboard and info btn
</commit_message>
<xml_diff>
--- a/docs/tasks-lambda.xlsx
+++ b/docs/tasks-lambda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\einav\clone_here\Lambda\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B757D9E9-693F-4B29-8B94-36E98EDAB1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BA528B-8CEC-4891-8916-5D2AC71D3DC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3247" yWindow="2138" windowWidth="16200" windowHeight="9307" xr2:uid="{64494733-B6F9-48B6-9193-F7C7FF2B1841}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>הוספה של אופציה להוסיף שאלות כלליות (לאו דווקא ממבחן) - רבות ברירה, שאלות פתוחות</t>
   </si>
@@ -345,6 +345,12 @@
   </si>
   <si>
     <t>מערכת יותר ברורה לשאלות האמריקאיות</t>
+  </si>
+  <si>
+    <t>פחות nodes ברקע בmobile</t>
+  </si>
+  <si>
+    <t>delete account option</t>
   </si>
 </sst>
 </file>
@@ -751,7 +757,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ABCB3E3-AEE1-47E5-A283-0150B72CF279}">
-  <dimension ref="A1:O98"/>
+  <dimension ref="A1:O100"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.45">
@@ -1558,6 +1564,22 @@
         <v>102</v>
       </c>
     </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A99" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B99" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A100" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B100" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
meta data - web description
</commit_message>
<xml_diff>
--- a/docs/tasks-lambda.xlsx
+++ b/docs/tasks-lambda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\einav\clone_here\Lambda\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2887364D-0062-4DB7-9031-4DD06C5C497C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2C8FF66-84E5-4211-95E8-85C21E7FFF42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{64494733-B6F9-48B6-9193-F7C7FF2B1841}"/>
   </bookViews>
@@ -1629,7 +1629,7 @@
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A105" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B105" t="s">
         <v>109</v>

</xml_diff>

<commit_message>
mobile: community btn, delay, fewer nodes, flashcards width
</commit_message>
<xml_diff>
--- a/docs/tasks-lambda.xlsx
+++ b/docs/tasks-lambda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\einav\clone_here\Lambda\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2C8FF66-84E5-4211-95E8-85C21E7FFF42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D50332D-24D4-4BA1-ACF6-6E5BE94DFD74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{64494733-B6F9-48B6-9193-F7C7FF2B1841}"/>
   </bookViews>
@@ -1581,7 +1581,7 @@
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A99" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B99" t="s">
         <v>102</v>
@@ -1605,7 +1605,7 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A102" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B102" t="s">
         <v>106</v>
@@ -1613,7 +1613,7 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A103" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B103" t="s">
         <v>105</v>
@@ -1621,7 +1621,7 @@
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A104" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B104" t="s">
         <v>108</v>

</xml_diff>

<commit_message>
fix delay in mobile flashcards
</commit_message>
<xml_diff>
--- a/docs/tasks-lambda.xlsx
+++ b/docs/tasks-lambda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\einav\clone_here\Lambda\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29206819-EF5F-4022-9076-F76E786AC023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5492F7B5-20D2-4304-B121-674D9CA488AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{64494733-B6F9-48B6-9193-F7C7FF2B1841}"/>
   </bookViews>
@@ -1668,7 +1668,7 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A107" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B107" t="s">
         <v>111</v>
@@ -1676,7 +1676,7 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A108" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B108" t="s">
         <v>112</v>

</xml_diff>